<commit_message>
Compute some totals for some columns
</commit_message>
<xml_diff>
--- a/Info_W1/Analysis 1/output/sku_monthly_quantities.xlsx
+++ b/Info_W1/Analysis 1/output/sku_monthly_quantities.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ULB\MA2\Q2\Supply Chain Performance Analytics\Business-Case-NutryWell\Info_W1\Analysis 1\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{924F899E-CDF9-4F5A-9494-2025423EDCC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DFFEF97-E97C-4242-B209-017EA4ADDB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="E-commerce" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -97,7 +97,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -128,12 +128,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,7 +494,7 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>